<commit_message>
Refactor course plans for Ljud- och musikproduktion
- Removed quality notes from multiple course plans (GLP2QD, GLP2QU, GLP2UG, GLP2VS, GLP2WB, GLP2WC, LP1054, LP1064, LP1065, LP1072, LP1075, LP1076, LP1080, LP2009, LP2010, LP2012, LP2013, PE1023).
- Updated various Excel analysis files related to grading, examination forms, phrasing consistency, and other quality metrics.
</commit_message>
<xml_diff>
--- a/vault-dalarna-university/03 IKS/Analys/Bloom-taxonomi.xlsx
+++ b/vault-dalarna-university/03 IKS/Analys/Bloom-taxonomi.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Bloom-taxonomi" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Bloom-taxonomi'!$A$1:$G$68</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Bloom-taxonomi'!$A$1:$G$67</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G68"/>
+  <dimension ref="A1:G67"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1419,7 +1419,7 @@
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>GLP234</t>
+          <t>GLP2MU</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1429,7 +1429,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>2018-05-21</t>
+          <t>2021-03-02</t>
         </is>
       </c>
       <c r="D29" t="inlineStr"/>
@@ -1440,19 +1440,19 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Grundkurs domineras av värdera/skapa; fördelning [0,0,0,0,1,2]</t>
+          <t>Grundkurs domineras av värdera/skapa; fördelning [0,1,0,0,0,2]</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GLP234</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GLP2MU</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>GLP2MU</t>
+          <t>GLP2QX</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1462,7 +1462,7 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>2021-03-02</t>
+          <t>2021-08-20</t>
         </is>
       </c>
       <c r="D30" t="inlineStr"/>
@@ -1478,14 +1478,14 @@
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GLP2MU</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GLP2QX</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>GLP2QX</t>
+          <t>LP1071</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1495,10 +1495,14 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>2021-08-20</t>
-        </is>
-      </c>
-      <c r="D31" t="inlineStr"/>
+          <t>2015-12-10</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>2020-07-02</t>
+        </is>
+      </c>
       <c r="E31" t="inlineStr">
         <is>
           <t>Hög verbnivå för grundkurs</t>
@@ -1506,36 +1510,32 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>Grundkurs domineras av värdera/skapa; fördelning [0,1,0,0,0,2]</t>
+          <t>Grundkurs domineras av värdera/skapa; fördelning [0,0,0,0,1,2]</t>
         </is>
       </c>
       <c r="G31" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GLP2QX</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=LP1071</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>LP1071</t>
+          <t>GMN3EZ</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>LPU</t>
+          <t>MPR</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>2015-12-10</t>
-        </is>
-      </c>
-      <c r="D32" t="inlineStr">
-        <is>
-          <t>2020-07-02</t>
-        </is>
-      </c>
+          <t>2025-02-06</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr"/>
       <c r="E32" t="inlineStr">
         <is>
           <t>Hög verbnivå för grundkurs</t>
@@ -1543,52 +1543,56 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>Grundkurs domineras av värdera/skapa; fördelning [0,0,0,0,1,2]</t>
+          <t>Grundkurs domineras av värdera/skapa; fördelning [1,0,0,1,0,3]</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=LP1071</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMN3EZ</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>GMN3EZ</t>
+          <t>NA1003</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>MPR</t>
+          <t>NAA</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>2025-02-06</t>
-        </is>
-      </c>
-      <c r="D33" t="inlineStr"/>
+          <t>2006-12-06</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>2009-03-05</t>
+        </is>
+      </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Hög verbnivå för grundkurs</t>
+          <t>Okänt ledande verb</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>Grundkurs domineras av värdera/skapa; fördelning [1,0,0,1,0,3]</t>
+          <t>5 av 10 bullets har okänt ledande verb</t>
         </is>
       </c>
       <c r="G33" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMN3EZ</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=NA1003</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>NA1003</t>
+          <t>NA1026</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -1598,14 +1602,10 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>2006-12-06</t>
-        </is>
-      </c>
-      <c r="D34" t="inlineStr">
-        <is>
-          <t>2009-03-05</t>
-        </is>
-      </c>
+          <t>2009-10-19</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr"/>
       <c r="E34" t="inlineStr">
         <is>
           <t>Okänt ledande verb</t>
@@ -1613,19 +1613,19 @@
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>5 av 10 bullets har okänt ledande verb</t>
+          <t>6 av 10 bullets har okänt ledande verb</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=NA1003</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=NA1026</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>NA1026</t>
+          <t>NA1027</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -1638,7 +1638,11 @@
           <t>2009-10-19</t>
         </is>
       </c>
-      <c r="D35" t="inlineStr"/>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>2013-03-07</t>
+        </is>
+      </c>
       <c r="E35" t="inlineStr">
         <is>
           <t>Okänt ledande verb</t>
@@ -1646,19 +1650,19 @@
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>6 av 10 bullets har okänt ledande verb</t>
+          <t>4 av 10 bullets har okänt ledande verb</t>
         </is>
       </c>
       <c r="G35" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=NA1026</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=NA1027</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>NA1027</t>
+          <t>NA3001</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -1668,14 +1672,10 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>2009-10-19</t>
-        </is>
-      </c>
-      <c r="D36" t="inlineStr">
-        <is>
-          <t>2013-03-07</t>
-        </is>
-      </c>
+          <t>2006-12-06</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr"/>
       <c r="E36" t="inlineStr">
         <is>
           <t>Okänt ledande verb</t>
@@ -1688,14 +1688,14 @@
       </c>
       <c r="G36" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=NA1027</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=NA3001</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>NA3001</t>
+          <t>NA3007</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -1705,30 +1705,34 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>2006-12-06</t>
-        </is>
-      </c>
-      <c r="D37" t="inlineStr"/>
+          <t>2007-09-05</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>2008-02-07</t>
+        </is>
+      </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Okänt ledande verb</t>
+          <t>Låg verbnivå för avancerad kurs</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>4 av 10 bullets har okänt ledande verb</t>
+          <t>Avancerad kurs utan analysera/värdera/skapa-verb; fördelning [0,7,1,0,0,0]</t>
         </is>
       </c>
       <c r="G37" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=NA3001</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=NA3007</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>NA3007</t>
+          <t>NA3008</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -1741,101 +1745,101 @@
           <t>2007-09-05</t>
         </is>
       </c>
-      <c r="D38" t="inlineStr">
-        <is>
-          <t>2008-02-07</t>
-        </is>
-      </c>
+      <c r="D38" t="inlineStr"/>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Låg verbnivå för avancerad kurs</t>
+          <t>Okänt ledande verb</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>Avancerad kurs utan analysera/värdera/skapa-verb; fördelning [0,7,1,0,0,0]</t>
+          <t>4 av 4 bullets har okänt ledande verb</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=NA3007</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=NA3008</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>NA3008</t>
+          <t>PE1069</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>NAA</t>
+          <t>PEA</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>2007-09-05</t>
-        </is>
-      </c>
-      <c r="D39" t="inlineStr"/>
+          <t>2013-11-11</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>2014-01-24</t>
+        </is>
+      </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Okänt ledande verb</t>
+          <t>Hög verbnivå för grundkurs</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>4 av 4 bullets har okänt ledande verb</t>
+          <t>Grundkurs domineras av värdera/skapa; fördelning [1,0,0,0,0,2]</t>
         </is>
       </c>
       <c r="G39" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=NA3008</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=PE1069</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>PE1069</t>
+          <t>APG24E</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>PEA</t>
+          <t>PGA</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>2013-11-11</t>
+          <t>2020-02-24</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>2014-01-24</t>
+          <t>2020-06-23</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Hög verbnivå för grundkurs</t>
+          <t>Låg verbnivå för avancerad kurs</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>Grundkurs domineras av värdera/skapa; fördelning [1,0,0,0,0,2]</t>
+          <t>Avancerad kurs utan analysera/värdera/skapa-verb; fördelning [7,0,0,0,0,0]</t>
         </is>
       </c>
       <c r="G40" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=PE1069</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=APG24E</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>APG24E</t>
+          <t>APG24S</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -1845,14 +1849,10 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>2020-02-24</t>
-        </is>
-      </c>
-      <c r="D41" t="inlineStr">
-        <is>
-          <t>2020-06-23</t>
-        </is>
-      </c>
+          <t>2020-02-25</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr"/>
       <c r="E41" t="inlineStr">
         <is>
           <t>Låg verbnivå för avancerad kurs</t>
@@ -1860,19 +1860,19 @@
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>Avancerad kurs utan analysera/värdera/skapa-verb; fördelning [7,0,0,0,0,0]</t>
+          <t>Avancerad kurs utan analysera/värdera/skapa-verb; fördelning [3,0,0,0,0,0]</t>
         </is>
       </c>
       <c r="G41" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=APG24E</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=APG24S</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>APG24S</t>
+          <t>APG27T</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1882,7 +1882,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>2020-02-25</t>
+          <t>2022-02-25</t>
         </is>
       </c>
       <c r="D42" t="inlineStr"/>
@@ -1893,19 +1893,19 @@
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>Avancerad kurs utan analysera/värdera/skapa-verb; fördelning [3,0,0,0,0,0]</t>
+          <t>Avancerad kurs utan analysera/värdera/skapa-verb; fördelning [5,0,0,0,0,0]</t>
         </is>
       </c>
       <c r="G42" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=APG24S</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=APG27T</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>APG27T</t>
+          <t>APG27U</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -1915,7 +1915,7 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>2022-02-25</t>
+          <t>2022-03-01</t>
         </is>
       </c>
       <c r="D43" t="inlineStr"/>
@@ -1926,19 +1926,19 @@
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>Avancerad kurs utan analysera/värdera/skapa-verb; fördelning [5,0,0,0,0,0]</t>
+          <t>Avancerad kurs utan analysera/värdera/skapa-verb; fördelning [7,0,0,0,0,0]</t>
         </is>
       </c>
       <c r="G43" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=APG27T</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=APG27U</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>APG27U</t>
+          <t>APG27Z</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -1948,7 +1948,7 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>2022-03-01</t>
+          <t>2022-06-13</t>
         </is>
       </c>
       <c r="D44" t="inlineStr"/>
@@ -1959,19 +1959,19 @@
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>Avancerad kurs utan analysera/värdera/skapa-verb; fördelning [7,0,0,0,0,0]</t>
+          <t>Avancerad kurs utan analysera/värdera/skapa-verb; fördelning [12,0,0,0,0,0]</t>
         </is>
       </c>
       <c r="G44" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=APG27U</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=APG27Z</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>APG27Z</t>
+          <t>APG282</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -1992,19 +1992,19 @@
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>Avancerad kurs utan analysera/värdera/skapa-verb; fördelning [12,0,0,0,0,0]</t>
+          <t>Avancerad kurs utan analysera/värdera/skapa-verb; fördelning [8,0,0,0,0,0]</t>
         </is>
       </c>
       <c r="G45" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=APG27Z</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=APG282</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>APG282</t>
+          <t>APG28B</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -2014,7 +2014,7 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>2022-06-13</t>
+          <t>2022-11-21</t>
         </is>
       </c>
       <c r="D46" t="inlineStr"/>
@@ -2025,19 +2025,19 @@
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>Avancerad kurs utan analysera/värdera/skapa-verb; fördelning [8,0,0,0,0,0]</t>
+          <t>Avancerad kurs utan analysera/värdera/skapa-verb; fördelning [10,0,0,0,0,0]</t>
         </is>
       </c>
       <c r="G46" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=APG282</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=APG28B</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>APG28B</t>
+          <t>APG28M</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -2047,7 +2047,7 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>2022-11-21</t>
+          <t>2022-12-12</t>
         </is>
       </c>
       <c r="D47" t="inlineStr"/>
@@ -2058,19 +2058,19 @@
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>Avancerad kurs utan analysera/värdera/skapa-verb; fördelning [10,0,0,0,0,0]</t>
+          <t>Avancerad kurs utan analysera/värdera/skapa-verb; fördelning [5,0,0,0,0,0]</t>
         </is>
       </c>
       <c r="G47" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=APG28B</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=APG28M</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>APG28M</t>
+          <t>APG28R</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -2080,7 +2080,7 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>2022-12-12</t>
+          <t>2023-01-24</t>
         </is>
       </c>
       <c r="D48" t="inlineStr"/>
@@ -2091,19 +2091,19 @@
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>Avancerad kurs utan analysera/värdera/skapa-verb; fördelning [5,0,0,0,0,0]</t>
+          <t>Avancerad kurs utan analysera/värdera/skapa-verb; fördelning [9,0,0,0,0,0]</t>
         </is>
       </c>
       <c r="G48" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=APG28M</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=APG28R</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>APG28R</t>
+          <t>APG28S</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -2129,14 +2129,14 @@
       </c>
       <c r="G49" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=APG28R</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=APG28S</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>APG28S</t>
+          <t>GPG3EV</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -2146,30 +2146,30 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>2023-01-24</t>
+          <t>2025-02-05</t>
         </is>
       </c>
       <c r="D50" t="inlineStr"/>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Låg verbnivå för avancerad kurs</t>
+          <t>Okänt ledande verb</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>Avancerad kurs utan analysera/värdera/skapa-verb; fördelning [9,0,0,0,0,0]</t>
+          <t>3 av 13 bullets har okänt ledande verb</t>
         </is>
       </c>
       <c r="G50" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=APG28S</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GPG3EV</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>GPG3EV</t>
+          <t>PG3069</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -2179,10 +2179,14 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>2025-02-05</t>
-        </is>
-      </c>
-      <c r="D51" t="inlineStr"/>
+          <t>2017-10-26</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>2018-04-12</t>
+        </is>
+      </c>
       <c r="E51" t="inlineStr">
         <is>
           <t>Okänt ledande verb</t>
@@ -2190,56 +2194,52 @@
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>3 av 13 bullets har okänt ledande verb</t>
+          <t>3 av 5 bullets har okänt ledande verb</t>
         </is>
       </c>
       <c r="G51" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GPG3EV</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=PG3069</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>PG3069</t>
+          <t>ARK29H</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>PGA</t>
+          <t>RKA</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>2017-10-26</t>
-        </is>
-      </c>
-      <c r="D52" t="inlineStr">
-        <is>
-          <t>2018-04-12</t>
-        </is>
-      </c>
+          <t>2023-09-08</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr"/>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Okänt ledande verb</t>
+          <t>Låg verbnivå för avancerad kurs</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>3 av 5 bullets har okänt ledande verb</t>
+          <t>Avancerad kurs utan analysera/värdera/skapa-verb; fördelning [0,3,0,0,0,0]</t>
         </is>
       </c>
       <c r="G52" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=PG3069</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ARK29H</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t>ARK29H</t>
+          <t>GRK2Q5</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -2249,40 +2249,40 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>2023-09-08</t>
+          <t>2021-05-24</t>
         </is>
       </c>
       <c r="D53" t="inlineStr"/>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Låg verbnivå för avancerad kurs</t>
+          <t>Okänt ledande verb</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>Avancerad kurs utan analysera/värdera/skapa-verb; fördelning [0,3,0,0,0,0]</t>
+          <t>3 av 11 bullets har okänt ledande verb</t>
         </is>
       </c>
       <c r="G53" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ARK29H</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GRK2Q5</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>GRK2Q5</t>
+          <t>RV1009</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>RKA</t>
+          <t>RVA</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>2021-05-24</t>
+          <t>2007-01-10</t>
         </is>
       </c>
       <c r="D54" t="inlineStr"/>
@@ -2293,19 +2293,19 @@
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>3 av 11 bullets har okänt ledande verb</t>
+          <t>3 av 5 bullets har okänt ledande verb</t>
         </is>
       </c>
       <c r="G54" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GRK2Q5</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=RV1009</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
         <is>
-          <t>RV1009</t>
+          <t>RV1015</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -2315,7 +2315,7 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>2007-01-10</t>
+          <t>2007-04-04</t>
         </is>
       </c>
       <c r="D55" t="inlineStr"/>
@@ -2326,19 +2326,19 @@
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>3 av 5 bullets har okänt ledande verb</t>
+          <t>3 av 6 bullets har okänt ledande verb</t>
         </is>
       </c>
       <c r="G55" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=RV1009</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=RV1015</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>RV1015</t>
+          <t>RV1037</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -2348,7 +2348,7 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>2007-04-04</t>
+          <t>2008-06-10</t>
         </is>
       </c>
       <c r="D56" t="inlineStr"/>
@@ -2364,14 +2364,14 @@
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=RV1015</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=RV1037</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
         <is>
-          <t>RV1037</t>
+          <t>RV1043</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -2381,7 +2381,7 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>2008-06-10</t>
+          <t>2012-03-08</t>
         </is>
       </c>
       <c r="D57" t="inlineStr"/>
@@ -2392,135 +2392,139 @@
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>3 av 6 bullets har okänt ledande verb</t>
+          <t>4 av 11 bullets har okänt ledande verb</t>
         </is>
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=RV1037</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=RV1043</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>RV1043</t>
+          <t>ASK22L</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>RVA</t>
+          <t>SKA</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>2012-03-08</t>
-        </is>
-      </c>
-      <c r="D58" t="inlineStr"/>
+          <t>2018-11-15</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>2019-08-20</t>
+        </is>
+      </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>Okänt ledande verb</t>
+          <t>Låg verbnivå för avancerad kurs</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>4 av 11 bullets har okänt ledande verb</t>
+          <t>Avancerad kurs utan analysera/värdera/skapa-verb; fördelning [6,0,2,0,0,0]</t>
         </is>
       </c>
       <c r="G58" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=RV1043</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASK22L</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
         <is>
-          <t>ASK22L</t>
+          <t>GSO2PL</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>SKA</t>
+          <t>SOA</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>2018-11-15</t>
-        </is>
-      </c>
-      <c r="D59" t="inlineStr">
-        <is>
-          <t>2019-08-20</t>
-        </is>
-      </c>
+          <t>2021-04-15</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr"/>
       <c r="E59" t="inlineStr">
         <is>
-          <t>Låg verbnivå för avancerad kurs</t>
+          <t>Okänt ledande verb</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>Avancerad kurs utan analysera/värdera/skapa-verb; fördelning [6,0,2,0,0,0]</t>
+          <t>3 av 10 bullets har okänt ledande verb</t>
         </is>
       </c>
       <c r="G59" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASK22L</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSO2PL</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>GSO2PL</t>
+          <t>ATR26B</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>SOA</t>
+          <t>TRU</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>2021-04-15</t>
+          <t>2020-10-15</t>
         </is>
       </c>
       <c r="D60" t="inlineStr"/>
       <c r="E60" t="inlineStr">
         <is>
-          <t>Okänt ledande verb</t>
+          <t>Låg verbnivå för avancerad kurs</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>3 av 10 bullets har okänt ledande verb</t>
+          <t>Avancerad kurs utan analysera/värdera/skapa-verb; fördelning [4,1,1,0,0,0]</t>
         </is>
       </c>
       <c r="G60" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSO2PL</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ATR26B</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
         <is>
-          <t>ATR26B</t>
+          <t>AS3002</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>TRU</t>
+          <t>UVX</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>2020-10-15</t>
-        </is>
-      </c>
-      <c r="D61" t="inlineStr"/>
+          <t>2014-12-10</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>2023-03-06</t>
+        </is>
+      </c>
       <c r="E61" t="inlineStr">
         <is>
           <t>Låg verbnivå för avancerad kurs</t>
@@ -2528,19 +2532,19 @@
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>Avancerad kurs utan analysera/värdera/skapa-verb; fördelning [4,1,1,0,0,0]</t>
+          <t>Avancerad kurs utan analysera/värdera/skapa-verb; fördelning [3,0,0,0,0,0]</t>
         </is>
       </c>
       <c r="G61" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ATR26B</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AS3002</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>AS3002</t>
+          <t>AS3003</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -2565,19 +2569,19 @@
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>Avancerad kurs utan analysera/värdera/skapa-verb; fördelning [3,0,0,0,0,0]</t>
+          <t>Avancerad kurs utan analysera/värdera/skapa-verb; fördelning [1,1,0,0,0,0]</t>
         </is>
       </c>
       <c r="G62" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AS3002</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AS3003</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
         <is>
-          <t>AS3003</t>
+          <t>AS3004</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -2587,7 +2591,7 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>2014-12-10</t>
+          <t>2015-06-17</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
@@ -2602,19 +2606,19 @@
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>Avancerad kurs utan analysera/värdera/skapa-verb; fördelning [1,1,0,0,0,0]</t>
+          <t>Avancerad kurs utan analysera/värdera/skapa-verb; fördelning [3,0,0,0,0,0]</t>
         </is>
       </c>
       <c r="G63" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AS3003</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AS3004</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>AS3004</t>
+          <t>AS3008</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -2624,14 +2628,10 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>2015-06-17</t>
-        </is>
-      </c>
-      <c r="D64" t="inlineStr">
-        <is>
-          <t>2023-03-06</t>
-        </is>
-      </c>
+          <t>2015-10-05</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr"/>
       <c r="E64" t="inlineStr">
         <is>
           <t>Låg verbnivå för avancerad kurs</t>
@@ -2639,19 +2639,19 @@
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>Avancerad kurs utan analysera/värdera/skapa-verb; fördelning [3,0,0,0,0,0]</t>
+          <t>Avancerad kurs utan analysera/värdera/skapa-verb; fördelning [4,0,0,0,0,0]</t>
         </is>
       </c>
       <c r="G64" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AS3004</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AS3008</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
         <is>
-          <t>AS3008</t>
+          <t>AS3012</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -2677,14 +2677,14 @@
       </c>
       <c r="G65" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AS3008</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AS3012</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>AS3012</t>
+          <t>AS4001</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -2694,7 +2694,7 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>2015-10-05</t>
+          <t>2016-05-03</t>
         </is>
       </c>
       <c r="D66" t="inlineStr"/>
@@ -2705,19 +2705,19 @@
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>Avancerad kurs utan analysera/värdera/skapa-verb; fördelning [4,0,0,0,0,0]</t>
+          <t>Avancerad kurs utan analysera/värdera/skapa-verb; fördelning [1,0,1,0,0,0]</t>
         </is>
       </c>
       <c r="G66" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AS3012</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AS4001</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
         <is>
-          <t>AS4001</t>
+          <t>AS4003</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -2738,50 +2738,17 @@
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>Avancerad kurs utan analysera/värdera/skapa-verb; fördelning [1,0,1,0,0,0]</t>
+          <t>Avancerad kurs utan analysera/värdera/skapa-verb; fördelning [3,0,0,0,0,0]</t>
         </is>
       </c>
       <c r="G67" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AS4001</t>
-        </is>
-      </c>
-    </row>
-    <row r="68">
-      <c r="A68" s="2" t="inlineStr">
-        <is>
-          <t>AS4003</t>
-        </is>
-      </c>
-      <c r="B68" t="inlineStr">
-        <is>
-          <t>UVX</t>
-        </is>
-      </c>
-      <c r="C68" t="inlineStr">
-        <is>
-          <t>2016-05-03</t>
-        </is>
-      </c>
-      <c r="D68" t="inlineStr"/>
-      <c r="E68" t="inlineStr">
-        <is>
-          <t>Låg verbnivå för avancerad kurs</t>
-        </is>
-      </c>
-      <c r="F68" t="inlineStr">
-        <is>
-          <t>Avancerad kurs utan analysera/värdera/skapa-verb; fördelning [3,0,0,0,0,0]</t>
-        </is>
-      </c>
-      <c r="G68" s="2" t="inlineStr">
-        <is>
           <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AS4003</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G68"/>
+  <autoFilter ref="A1:G67"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G2" r:id="rId2"/>
@@ -2915,8 +2882,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G66" r:id="rId130"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A67" r:id="rId131"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G67" r:id="rId132"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A68" r:id="rId133"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G68" r:id="rId134"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>